<commit_message>
commit inicial na develop
</commit_message>
<xml_diff>
--- a/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
+++ b/graficos_tabelas/preliminares/Tabela_resumo_thetas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6e8fc6e241c731ae/UFABC/Dissertação/volatilidade-IBOV-GPR/Impacto-geopolitico-ibovespa/graficos_tabelas/preliminares/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1163" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31F92FE9-3007-424B-B2DF-CF2A3E88C64C}"/>
+  <xr:revisionPtr revIDLastSave="1172" documentId="11_F25DC773A252ABDACC1048C0F11B46C65ADE58EB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E13DC02-2EB5-4BAF-9389-F9F49483B1B0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IBOV" sheetId="1" r:id="rId1"/>
@@ -605,15 +605,6 @@
     <t>0.025</t>
   </si>
   <si>
-    <t>0.3810</t>
-  </si>
-  <si>
-    <t>0.195</t>
-  </si>
-  <si>
-    <t>-0.6530</t>
-  </si>
-  <si>
     <t>0.065</t>
   </si>
   <si>
@@ -1590,6 +1581,15 @@
   </si>
   <si>
     <t>0.541</t>
+  </si>
+  <si>
+    <t xml:space="preserve">−0,7113 </t>
+  </si>
+  <si>
+    <t>0.043</t>
+  </si>
+  <si>
+    <t>0.6730</t>
   </si>
 </sst>
 </file>
@@ -2178,22 +2178,22 @@
         <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2284,19 +2284,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>26</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>27</v>
@@ -2391,7 +2391,7 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -2431,16 +2431,16 @@
         <v>-101.75</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>87</v>
@@ -2451,19 +2451,19 @@
         <v>6</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>167</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>95</v>
@@ -2474,27 +2474,27 @@
         <v>7</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>167</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -2531,19 +2531,19 @@
         <v>5</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>137</v>
@@ -2554,19 +2554,19 @@
         <v>6</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>119</v>
@@ -2577,22 +2577,22 @@
         <v>7</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>100</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>107</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
@@ -3159,7 +3159,7 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="B57" s="9"/>
       <c r="C57" s="9"/>
@@ -3196,22 +3196,22 @@
         <v>7</v>
       </c>
       <c r="B59" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="F59" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="G59" s="1" t="s">
         <v>440</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
@@ -3219,7 +3219,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B61" s="9"/>
       <c r="C61" s="9"/>
@@ -3256,22 +3256,22 @@
         <v>7</v>
       </c>
       <c r="B63" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>507</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="E63" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="F63" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="D63" s="1" t="s">
+      <c r="G63" s="1" t="s">
         <v>511</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>513</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
@@ -3285,7 +3285,7 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B65" s="9"/>
       <c r="C65" s="9"/>
@@ -3330,7 +3330,7 @@
         <v>80</v>
       </c>
       <c r="K66" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3344,7 +3344,7 @@
         <v>12</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>7</v>
@@ -3353,19 +3353,19 @@
         <v>12</v>
       </c>
       <c r="G67" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="J67" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="H67" s="1" t="s">
+      <c r="K67" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>449</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3379,7 +3379,7 @@
         <v>6</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>7</v>
@@ -3388,19 +3388,19 @@
         <v>6</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>69</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -3414,7 +3414,7 @@
         <v>3</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>7</v>
@@ -3423,19 +3423,19 @@
         <v>3</v>
       </c>
       <c r="G69" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="J69" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="H69" s="1" t="s">
+      <c r="K69" s="1" t="s">
         <v>455</v>
-      </c>
-      <c r="I69" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -3449,7 +3449,7 @@
         <v>3</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>7</v>
@@ -3458,19 +3458,19 @@
         <v>1</v>
       </c>
       <c r="G70" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="J70" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="H70" s="1" t="s">
+      <c r="K70" s="1" t="s">
         <v>460</v>
-      </c>
-      <c r="I70" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="J70" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -3484,7 +3484,7 @@
         <v>12</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>7</v>
@@ -3493,19 +3493,19 @@
         <v>12</v>
       </c>
       <c r="G71" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="J71" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="H71" s="1" t="s">
+      <c r="K71" s="1" t="s">
         <v>465</v>
-      </c>
-      <c r="I71" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -3519,7 +3519,7 @@
         <v>6</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>7</v>
@@ -3528,19 +3528,19 @@
         <v>6</v>
       </c>
       <c r="G72" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="J72" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="H72" s="1" t="s">
+      <c r="K72" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="I72" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -3554,7 +3554,7 @@
         <v>3</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>7</v>
@@ -3563,19 +3563,19 @@
         <v>3</v>
       </c>
       <c r="G73" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="K73" s="1" t="s">
         <v>474</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -3589,7 +3589,7 @@
         <v>3</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>7</v>
@@ -3598,19 +3598,19 @@
         <v>1</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="J74" s="1" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="K74" s="1" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
   </sheetData>
@@ -3783,13 +3783,13 @@
         <v>45</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -3800,19 +3800,19 @@
         <v>64</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>65</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>66</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -3863,13 +3863,13 @@
         <v>49</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>51</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -3880,19 +3880,19 @@
         <v>-1190</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>67</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>68</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -4042,22 +4042,22 @@
         <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>45</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -4068,19 +4068,19 @@
         <v>64</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>65</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>66</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -4156,31 +4156,31 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="G9" s="5" t="s">
         <v>494</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="H9" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="I9" s="5" t="s">
         <v>496</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>497</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>498</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -4377,16 +4377,16 @@
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>192</v>
+        <v>519</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>167</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>194</v>
+        <v>517</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>518</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -4409,16 +4409,16 @@
         <v>6</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="J19" s="3" t="s">
         <v>195</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -4441,16 +4441,16 @@
         <v>3</v>
       </c>
       <c r="G20" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="J20" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -4473,16 +4473,16 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>91</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -4505,16 +4505,16 @@
         <v>12</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="J22" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -4537,16 +4537,16 @@
         <v>6</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -4569,16 +4569,16 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -4601,13 +4601,13 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>119</v>
@@ -4633,16 +4633,16 @@
         <v>12</v>
       </c>
       <c r="G26" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>226</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -4665,16 +4665,16 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="J27" s="3" t="s">
         <v>230</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -4697,16 +4697,16 @@
         <v>3</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="J28" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -4729,16 +4729,16 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="J29" s="5" t="s">
         <v>238</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -4816,13 +4816,13 @@
         <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -4833,24 +4833,24 @@
         <v>-1190</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>67</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -4895,28 +4895,28 @@
         <v>148</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>107</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -4924,33 +4924,33 @@
         <v>149</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>165</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>100</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -5014,13 +5014,13 @@
         <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>167</v>
@@ -5046,16 +5046,16 @@
         <v>6</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>258</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -5078,16 +5078,16 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -5110,16 +5110,16 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>265</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -5142,16 +5142,16 @@
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>119</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -5174,16 +5174,16 @@
         <v>6</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>100</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -5206,13 +5206,13 @@
         <v>3</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>100</v>
@@ -5238,16 +5238,16 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="J21" s="5" t="s">
         <v>277</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -5273,13 +5273,13 @@
         <v>-1339</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -5302,16 +5302,16 @@
         <v>6</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="J23" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -5334,13 +5334,13 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>137</v>
@@ -5366,16 +5366,16 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="I25" s="1" t="s">
         <v>97</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -5401,10 +5401,10 @@
         <v>-1519</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>111</v>
@@ -5430,16 +5430,16 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="H27" s="1" t="s">
         <v>173</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -5462,16 +5462,16 @@
         <v>3</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -5494,16 +5494,16 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="J29" s="5" t="s">
         <v>302</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -5574,7 +5574,7 @@
         <v>42</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>41</v>
@@ -5597,24 +5597,24 @@
         <v>61</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>62</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>63</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -5659,28 +5659,28 @@
         <v>148</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>338</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -5688,33 +5688,33 @@
         <v>149</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>346</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -5759,7 +5759,7 @@
         <v>80</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -5782,19 +5782,19 @@
         <v>12</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>352</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -5817,19 +5817,19 @@
         <v>6</v>
       </c>
       <c r="G15" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="J15" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>357</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -5852,19 +5852,19 @@
         <v>3</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="I16" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -5887,19 +5887,19 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="J17" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="K17" s="1" t="s">
         <v>366</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -5922,19 +5922,19 @@
         <v>12</v>
       </c>
       <c r="G18" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>370</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -5957,19 +5957,19 @@
         <v>6</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>140</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -5992,19 +5992,19 @@
         <v>3</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H20" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="K20" s="1" t="s">
         <v>378</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -6027,19 +6027,19 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="J21" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="K21" s="1" t="s">
         <v>383</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>385</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -6062,19 +6062,19 @@
         <v>12</v>
       </c>
       <c r="G22" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="J22" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="K22" s="1" t="s">
         <v>388</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>390</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -6097,19 +6097,19 @@
         <v>6</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>393</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -6132,19 +6132,19 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>105</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -6167,19 +6167,19 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="J25" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="K25" s="1" t="s">
         <v>402</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -6202,19 +6202,19 @@
         <v>12</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="K26" s="1" t="s">
         <v>407</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -6237,19 +6237,19 @@
         <v>6</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>145</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -6272,19 +6272,19 @@
         <v>3</v>
       </c>
       <c r="G28" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="K28" s="1" t="s">
         <v>415</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -6307,16 +6307,16 @@
         <v>1</v>
       </c>
       <c r="G29" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="J29" s="1" t="s">
         <v>419</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>422</v>
       </c>
       <c r="K29" s="1">
         <v>25110</v>
@@ -6386,22 +6386,22 @@
         <v>39</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>53</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>54</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -6412,24 +6412,24 @@
         <v>69</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>70</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>71</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -6474,62 +6474,62 @@
         <v>148</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="G8" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>429</v>
-      </c>
       <c r="I8" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>177</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="H9" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>433</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>434</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -6574,7 +6574,7 @@
         <v>80</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>